<commit_message>
Add comments and reviews
</commit_message>
<xml_diff>
--- a/Output/Correlation_exposure_table.xlsx
+++ b/Output/Correlation_exposure_table.xlsx
@@ -1,29 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10525"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11020"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uccl0-my.sharepoint.com/personal/estela_blanco_uc_cl/Documents/Contaminación_Malformaciones Congénitas/Pollution_Malformation_TEM/Output/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="11_54184E34035CA082CE475652F37BD2728A496552" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00F3A572-C90E-BC45-B1C8-669AE0787F6A}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="11_4892293001746D10E9270F82A2695E7C453E9B9F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F6C3B093-CACB-2B4A-B887-439B634CBDB5}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="1340" windowWidth="34560" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary_statistics_correlations" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Summary_statistics_correlations!$A$1:$K$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Summary_statistics_correlations!$A$1:$K$25</definedName>
   </definedNames>
   <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="33">
   <si>
     <t>period</t>
   </si>
@@ -37,7 +37,7 @@
     <t>max</t>
   </si>
   <si>
-    <t>Median (P25-P75)</t>
+    <t>Median (IQR, P75-P25)</t>
   </si>
   <si>
     <t>pct1</t>
@@ -61,7 +61,7 @@
     <t>Pre-conception</t>
   </si>
   <si>
-    <t>29.4 (13.8-54.6)</t>
+    <t>29.4 (40.8)</t>
   </si>
   <si>
     <t>PM2.5</t>
@@ -73,61 +73,55 @@
     <t>Trimester 1</t>
   </si>
   <si>
-    <t>32.1 (15.0-55.0)</t>
+    <t>31.0 (41.0)</t>
   </si>
   <si>
     <t>Trimester 2</t>
   </si>
   <si>
-    <t>34.5 (16.4-55.6)</t>
+    <t>34.5 (39.2)</t>
   </si>
   <si>
     <t>Trimester 3</t>
   </si>
   <si>
-    <t>31.5 (14.5-53.9)</t>
-  </si>
-  <si>
-    <t>0.4 (0.1-0.8)</t>
+    <t>32.3 (38.6)</t>
+  </si>
+  <si>
+    <t>0.4 (0.7)</t>
   </si>
   <si>
     <t>Levoglucosan</t>
   </si>
   <si>
-    <t>0.4 (0.2-0.9)</t>
-  </si>
-  <si>
     <t>K</t>
   </si>
   <si>
-    <t>0.5 (0.2-0.9)</t>
-  </si>
-  <si>
-    <t>0.5 (0.2-0.8)</t>
-  </si>
-  <si>
-    <t>46.0 (22.2-83.7)</t>
+    <t>0.5 (0.7)</t>
+  </si>
+  <si>
+    <t>46.0 (61.5)</t>
   </si>
   <si>
     <t>LUR</t>
   </si>
   <si>
-    <t>49.0 (23.4-85.5)</t>
-  </si>
-  <si>
-    <t>53.1 (25.0-87.9)</t>
-  </si>
-  <si>
-    <t>48.7 (22.9-83.2)</t>
-  </si>
-  <si>
-    <t>0.5 (0.1-0.8)</t>
-  </si>
-  <si>
-    <t>0.6 (0.2-1.2)</t>
-  </si>
-  <si>
-    <t>0.7 (0.3-1.2)</t>
+    <t>48.1 (63.0)</t>
+  </si>
+  <si>
+    <t>52.8 (62.2)</t>
+  </si>
+  <si>
+    <t>49.3 (59.6)</t>
+  </si>
+  <si>
+    <t>0.6 (0.9)</t>
+  </si>
+  <si>
+    <t>0.6 (1.0)</t>
+  </si>
+  <si>
+    <t>0.7 (0.9)</t>
   </si>
 </sst>
 </file>
@@ -483,14 +477,7 @@
   <dimension ref="A1:K25"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="12.83203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.83203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.1640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.1640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="5.6640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="16.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.2">
@@ -548,13 +535,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>0.11</v>
+        <v>0.17</v>
       </c>
       <c r="H2">
-        <v>-0.85</v>
+        <v>-0.84</v>
       </c>
       <c r="I2">
-        <v>0.03</v>
+        <v>-0.02</v>
       </c>
       <c r="J2" t="s">
         <v>13</v>
@@ -574,19 +561,19 @@
         <v>5.9</v>
       </c>
       <c r="D3">
-        <v>84.5</v>
+        <v>86.3</v>
       </c>
       <c r="E3" t="s">
         <v>16</v>
       </c>
       <c r="F3">
-        <v>0.11</v>
+        <v>0.17</v>
       </c>
       <c r="G3">
         <v>1</v>
       </c>
       <c r="H3">
-        <v>-0.02</v>
+        <v>0.03</v>
       </c>
       <c r="I3">
         <v>-0.84</v>
@@ -606,7 +593,7 @@
         <v>0</v>
       </c>
       <c r="C4">
-        <v>6</v>
+        <v>6.1</v>
       </c>
       <c r="D4">
         <v>82.9</v>
@@ -615,16 +602,16 @@
         <v>18</v>
       </c>
       <c r="F4">
-        <v>-0.85</v>
+        <v>-0.84</v>
       </c>
       <c r="G4">
-        <v>-0.02</v>
+        <v>0.03</v>
       </c>
       <c r="H4">
         <v>1</v>
       </c>
       <c r="I4">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="J4" t="s">
         <v>13</v>
@@ -638,25 +625,25 @@
         <v>19</v>
       </c>
       <c r="B5">
-        <v>70</v>
+        <v>42</v>
       </c>
       <c r="C5">
-        <v>4.5999999999999996</v>
+        <v>4.7</v>
       </c>
       <c r="D5">
-        <v>121.3</v>
+        <v>136</v>
       </c>
       <c r="E5" t="s">
         <v>20</v>
       </c>
       <c r="F5">
-        <v>0.03</v>
+        <v>-0.02</v>
       </c>
       <c r="G5">
         <v>-0.84</v>
       </c>
       <c r="H5">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="I5">
         <v>1</v>
@@ -688,13 +675,13 @@
         <v>1</v>
       </c>
       <c r="G6">
-        <v>0.06</v>
+        <v>0.12</v>
       </c>
       <c r="H6">
         <v>-0.89</v>
       </c>
       <c r="I6">
-        <v>-0.01</v>
+        <v>-0.06</v>
       </c>
       <c r="J6" t="s">
         <v>22</v>
@@ -720,13 +707,13 @@
         <v>21</v>
       </c>
       <c r="F7">
-        <v>0.06</v>
+        <v>0.12</v>
       </c>
       <c r="G7">
         <v>1</v>
       </c>
       <c r="H7">
-        <v>-0.08</v>
+        <v>-0.03</v>
       </c>
       <c r="I7">
         <v>-0.88</v>
@@ -758,13 +745,13 @@
         <v>-0.89</v>
       </c>
       <c r="G8">
-        <v>-0.08</v>
+        <v>-0.03</v>
       </c>
       <c r="H8">
         <v>1</v>
       </c>
       <c r="I8">
-        <v>0.02</v>
+        <v>-0.03</v>
       </c>
       <c r="J8" t="s">
         <v>22</v>
@@ -778,25 +765,25 @@
         <v>19</v>
       </c>
       <c r="B9">
-        <v>70</v>
+        <v>42</v>
       </c>
       <c r="C9">
         <v>0</v>
       </c>
       <c r="D9">
-        <v>1.8</v>
+        <v>2.2000000000000002</v>
       </c>
       <c r="E9" t="s">
         <v>21</v>
       </c>
       <c r="F9">
-        <v>-0.01</v>
+        <v>-0.06</v>
       </c>
       <c r="G9">
         <v>-0.88</v>
       </c>
       <c r="H9">
-        <v>0.02</v>
+        <v>-0.03</v>
       </c>
       <c r="I9">
         <v>1</v>
@@ -822,22 +809,22 @@
         <v>1.4</v>
       </c>
       <c r="E10" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="F10">
         <v>1</v>
       </c>
       <c r="G10">
-        <v>7.0000000000000007E-2</v>
+        <v>0.13</v>
       </c>
       <c r="H10">
         <v>-0.89</v>
       </c>
       <c r="I10">
-        <v>0</v>
+        <v>-0.05</v>
       </c>
       <c r="J10" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K10" t="s">
         <v>14</v>
@@ -857,22 +844,22 @@
         <v>1.4</v>
       </c>
       <c r="E11" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="F11">
-        <v>7.0000000000000007E-2</v>
+        <v>0.13</v>
       </c>
       <c r="G11">
         <v>1</v>
       </c>
       <c r="H11">
-        <v>-0.06</v>
+        <v>-0.01</v>
       </c>
       <c r="I11">
         <v>-0.88</v>
       </c>
       <c r="J11" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K11" t="s">
         <v>14</v>
@@ -892,22 +879,22 @@
         <v>1.4</v>
       </c>
       <c r="E12" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F12">
         <v>-0.89</v>
       </c>
       <c r="G12">
-        <v>-0.06</v>
+        <v>-0.01</v>
       </c>
       <c r="H12">
         <v>1</v>
       </c>
       <c r="I12">
-        <v>0.03</v>
+        <v>-0.03</v>
       </c>
       <c r="J12" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K12" t="s">
         <v>14</v>
@@ -918,31 +905,31 @@
         <v>19</v>
       </c>
       <c r="B13">
-        <v>70</v>
+        <v>42</v>
       </c>
       <c r="C13">
         <v>0.1</v>
       </c>
       <c r="D13">
-        <v>2.1</v>
+        <v>2.5</v>
       </c>
       <c r="E13" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="F13">
-        <v>0</v>
+        <v>-0.05</v>
       </c>
       <c r="G13">
         <v>-0.88</v>
       </c>
       <c r="H13">
-        <v>0.03</v>
+        <v>-0.03</v>
       </c>
       <c r="I13">
         <v>1</v>
       </c>
       <c r="J13" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K13" t="s">
         <v>14</v>
@@ -962,25 +949,25 @@
         <v>324.2</v>
       </c>
       <c r="E14" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="F14">
         <v>1</v>
       </c>
       <c r="G14">
-        <v>0.19</v>
+        <v>0.24</v>
       </c>
       <c r="H14">
-        <v>-0.69</v>
+        <v>-0.68</v>
       </c>
       <c r="I14">
-        <v>0.11</v>
+        <v>0.06</v>
       </c>
       <c r="J14" t="s">
         <v>13</v>
       </c>
       <c r="K14" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.2">
@@ -991,31 +978,31 @@
         <v>0</v>
       </c>
       <c r="C15">
-        <v>5.4</v>
+        <v>5.2</v>
       </c>
       <c r="D15">
-        <v>281.8</v>
+        <v>291.8</v>
       </c>
       <c r="E15" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="F15">
-        <v>0.19</v>
+        <v>0.24</v>
       </c>
       <c r="G15">
         <v>1</v>
       </c>
       <c r="H15">
-        <v>0.08</v>
+        <v>0.12</v>
       </c>
       <c r="I15">
-        <v>-0.69</v>
+        <v>-0.68</v>
       </c>
       <c r="J15" t="s">
         <v>13</v>
       </c>
       <c r="K15" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.2">
@@ -1029,28 +1016,28 @@
         <v>5.5</v>
       </c>
       <c r="D16">
-        <v>315</v>
+        <v>319.5</v>
       </c>
       <c r="E16" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="F16">
-        <v>-0.69</v>
+        <v>-0.68</v>
       </c>
       <c r="G16">
-        <v>0.08</v>
+        <v>0.12</v>
       </c>
       <c r="H16">
         <v>1</v>
       </c>
       <c r="I16">
-        <v>0.14000000000000001</v>
+        <v>0.1</v>
       </c>
       <c r="J16" t="s">
         <v>13</v>
       </c>
       <c r="K16" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.2">
@@ -1058,25 +1045,25 @@
         <v>19</v>
       </c>
       <c r="B17">
-        <v>70</v>
+        <v>42</v>
       </c>
       <c r="C17">
-        <v>5</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="D17">
-        <v>296.2</v>
+        <v>322.89999999999998</v>
       </c>
       <c r="E17" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F17">
-        <v>0.11</v>
+        <v>0.06</v>
       </c>
       <c r="G17">
-        <v>-0.69</v>
+        <v>-0.68</v>
       </c>
       <c r="H17">
-        <v>0.14000000000000001</v>
+        <v>0.1</v>
       </c>
       <c r="I17">
         <v>1</v>
@@ -1085,7 +1072,7 @@
         <v>13</v>
       </c>
       <c r="K17" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.2">
@@ -1108,19 +1095,19 @@
         <v>1</v>
       </c>
       <c r="G18">
-        <v>0.08</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="H18">
-        <v>-0.85</v>
+        <v>-0.84</v>
       </c>
       <c r="I18">
-        <v>0.01</v>
+        <v>-0.04</v>
       </c>
       <c r="J18" t="s">
         <v>22</v>
       </c>
       <c r="K18" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.2">
@@ -1140,13 +1127,13 @@
         <v>21</v>
       </c>
       <c r="F19">
-        <v>0.08</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="G19">
         <v>1</v>
       </c>
       <c r="H19">
-        <v>-0.04</v>
+        <v>0</v>
       </c>
       <c r="I19">
         <v>-0.84</v>
@@ -1155,7 +1142,7 @@
         <v>22</v>
       </c>
       <c r="K19" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.2">
@@ -1172,25 +1159,25 @@
         <v>1.6</v>
       </c>
       <c r="E20" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="F20">
-        <v>-0.85</v>
+        <v>-0.84</v>
       </c>
       <c r="G20">
-        <v>-0.04</v>
+        <v>0</v>
       </c>
       <c r="H20">
         <v>1</v>
       </c>
       <c r="I20">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="J20" t="s">
         <v>22</v>
       </c>
       <c r="K20" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.2">
@@ -1198,25 +1185,25 @@
         <v>19</v>
       </c>
       <c r="B21">
-        <v>70</v>
+        <v>42</v>
       </c>
       <c r="C21">
         <v>0</v>
       </c>
       <c r="D21">
-        <v>2</v>
+        <v>2.2000000000000002</v>
       </c>
       <c r="E21" t="s">
         <v>21</v>
       </c>
       <c r="F21">
-        <v>0.01</v>
+        <v>-0.04</v>
       </c>
       <c r="G21">
         <v>-0.84</v>
       </c>
       <c r="H21">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="I21">
         <v>1</v>
@@ -1225,7 +1212,7 @@
         <v>22</v>
       </c>
       <c r="K21" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.2">
@@ -1242,25 +1229,25 @@
         <v>4.2</v>
       </c>
       <c r="E22" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="F22">
         <v>1</v>
       </c>
       <c r="G22">
-        <v>0.12</v>
+        <v>0.18</v>
       </c>
       <c r="H22">
         <v>-0.78</v>
       </c>
       <c r="I22">
-        <v>0.06</v>
+        <v>0.01</v>
       </c>
       <c r="J22" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K22" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.2">
@@ -1277,25 +1264,25 @@
         <v>3.8</v>
       </c>
       <c r="E23" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="F23">
-        <v>0.12</v>
+        <v>0.18</v>
       </c>
       <c r="G23">
         <v>1</v>
       </c>
       <c r="H23">
-        <v>0.01</v>
+        <v>0.05</v>
       </c>
       <c r="I23">
         <v>-0.77</v>
       </c>
       <c r="J23" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K23" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.2">
@@ -1312,25 +1299,25 @@
         <v>3.9</v>
       </c>
       <c r="E24" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F24">
         <v>-0.78</v>
       </c>
       <c r="G24">
-        <v>0.01</v>
+        <v>0.05</v>
       </c>
       <c r="H24">
         <v>1</v>
       </c>
       <c r="I24">
-        <v>0.09</v>
+        <v>0.04</v>
       </c>
       <c r="J24" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K24" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.2">
@@ -1338,43 +1325,38 @@
         <v>19</v>
       </c>
       <c r="B25">
-        <v>70</v>
+        <v>42</v>
       </c>
       <c r="C25">
         <v>0.1</v>
       </c>
       <c r="D25">
-        <v>3.9</v>
+        <v>5</v>
       </c>
       <c r="E25" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="F25">
-        <v>0.06</v>
+        <v>0.01</v>
       </c>
       <c r="G25">
         <v>-0.77</v>
       </c>
       <c r="H25">
-        <v>0.09</v>
+        <v>0.04</v>
       </c>
       <c r="I25">
         <v>1</v>
       </c>
       <c r="J25" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K25" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K1" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:K25">
-      <sortCondition descending="1" ref="K1:K25"/>
-    </sortState>
-  </autoFilter>
+  <autoFilter ref="A1:K25" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>